<commit_message>
Updated Naca0012 3932 results onera l1 left
</commit_message>
<xml_diff>
--- a/001_POLIMO_CHAMPS/gridConvergence.xlsx
+++ b/001_POLIMO_CHAMPS/gridConvergence.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkzayni/Desktop/UNIVERSITY/POST_PROCESS/postProcessingData/001_POLIMO_CHAMPS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226C6C61-A950-5C48-828D-FA079A573D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6217A42F-A2AB-CA4C-A02B-661C6D9AAB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26940" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -603,6 +603,21 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -625,21 +640,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1054,23 +1054,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="35"/>
+      <c r="A2" s="40"/>
     </row>
     <row r="3" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="35"/>
+      <c r="A3" s="40"/>
     </row>
     <row r="4" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="40" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="35"/>
+      <c r="A5" s="40"/>
     </row>
     <row r="6" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1108,12 +1108,12 @@
       </c>
     </row>
     <row r="13" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="41" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="36"/>
+      <c r="A14" s="41"/>
     </row>
     <row r="15" spans="1:1" ht="22" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
@@ -1136,12 +1136,12 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="35" t="s">
+      <c r="A19" s="40" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="35"/>
+      <c r="A20" s="40"/>
     </row>
     <row r="21" spans="1:5" ht="22" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
@@ -1197,13 +1197,13 @@
       <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A31" s="35" t="s">
+      <c r="A31" s="40" t="s">
         <v>25</v>
       </c>
       <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="35"/>
+      <c r="A32" s="40"/>
       <c r="E32" s="4"/>
     </row>
     <row r="33" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1266,12 +1266,12 @@
       <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="35" t="s">
+      <c r="A43" s="40" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="35"/>
+      <c r="A44" s="40"/>
       <c r="E44" s="4"/>
     </row>
     <row r="45" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1335,12 +1335,12 @@
       <c r="E54" s="4"/>
     </row>
     <row r="55" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="35" t="s">
+      <c r="A55" s="40" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="35"/>
+      <c r="A56" s="40"/>
       <c r="E56" s="4"/>
     </row>
     <row r="57" spans="1:5" ht="22" x14ac:dyDescent="0.2">
@@ -1448,12 +1448,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:1024" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
@@ -6638,12 +6638,12 @@
       <c r="AMJ7" s="10"/>
     </row>
     <row r="8" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
+      <c r="B8" s="42"/>
+      <c r="C8" s="42"/>
+      <c r="D8" s="42"/>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="J8" s="7"/>
@@ -11842,12 +11842,12 @@
       <c r="AMJ14" s="10"/>
     </row>
     <row r="15" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="42" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="J15" s="7"/>
@@ -17046,12 +17046,12 @@
       <c r="AMJ21" s="10"/>
     </row>
     <row r="22" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="42" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
+      <c r="B22" s="42"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
       <c r="G22" s="7"/>
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
@@ -22256,12 +22256,12 @@
       <c r="R29" s="7"/>
     </row>
     <row r="30" spans="1:1024" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
@@ -23284,12 +23284,12 @@
       <c r="AMJ30" s="9"/>
     </row>
     <row r="31" spans="1:1024" ht="27" x14ac:dyDescent="0.2">
-      <c r="A31" s="38" t="s">
+      <c r="A31" s="43" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="38"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43"/>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -23733,12 +23733,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="42"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="47"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
@@ -23837,12 +23837,12 @@
       <c r="O7" s="10"/>
     </row>
     <row r="8" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="42"/>
+      <c r="B8" s="46"/>
+      <c r="C8" s="46"/>
+      <c r="D8" s="47"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10"/>
       <c r="I8" s="10"/>
@@ -23961,12 +23961,12 @@
       <c r="O14" s="10"/>
     </row>
     <row r="15" spans="1:18" ht="27" x14ac:dyDescent="0.2">
-      <c r="A15" s="40" t="s">
+      <c r="A15" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="42"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="47"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
@@ -24101,12 +24101,12 @@
       <c r="O21" s="10"/>
     </row>
     <row r="22" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="45" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="41"/>
-      <c r="C22" s="41"/>
-      <c r="D22" s="42"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="47"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
       <c r="I22" s="10"/>
@@ -24247,12 +24247,12 @@
       <c r="O29" s="10"/>
     </row>
     <row r="30" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A30" s="39" t="s">
+      <c r="A30" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
+      <c r="B30" s="44"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
@@ -24263,12 +24263,12 @@
       <c r="O30" s="10"/>
     </row>
     <row r="31" spans="1:15" ht="27" x14ac:dyDescent="0.2">
-      <c r="A31" s="39" t="s">
+      <c r="A31" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="B31" s="39"/>
-      <c r="C31" s="39"/>
-      <c r="D31" s="39"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
@@ -24738,65 +24738,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="27" x14ac:dyDescent="0.2">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
     </row>
     <row r="2" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
     </row>
     <row r="3" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47" t="s">
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47" t="s">
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
       <c r="Q3" s="19"/>
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
@@ -24853,27 +24853,45 @@
       <c r="A5" s="20">
         <v>1</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
+      <c r="B5" s="10">
+        <v>2.3608587888E-2</v>
+      </c>
+      <c r="C5" s="11">
+        <v>2.1613235168999999E-2</v>
+      </c>
+      <c r="D5" s="11">
+        <v>1.7348326136E-3</v>
+      </c>
       <c r="E5" s="21">
         <v>7.3890000000000002</v>
       </c>
       <c r="F5" s="20">
         <v>1</v>
       </c>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="16"/>
+      <c r="G5" s="11">
+        <v>1.1920214284999999E-2</v>
+      </c>
+      <c r="H5" s="11">
+        <v>1.0892186381999999E-2</v>
+      </c>
+      <c r="I5" s="16">
+        <v>8.9357825413999997E-4</v>
+      </c>
       <c r="J5" s="23">
         <v>5.6689999999999996</v>
       </c>
       <c r="K5" s="20">
         <v>1</v>
       </c>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
+      <c r="L5" s="11">
+        <v>1.1920214284999999E-2</v>
+      </c>
+      <c r="M5" s="11">
+        <v>1.0892188019E-2</v>
+      </c>
+      <c r="N5" s="11">
+        <v>8.9357825413999997E-4</v>
+      </c>
       <c r="O5" s="20">
         <v>5.6689999999999996</v>
       </c>
@@ -24886,27 +24904,45 @@
       <c r="A6" s="20">
         <v>2</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="16"/>
+      <c r="B6" s="11">
+        <v>9.2435112291000002E-2</v>
+      </c>
+      <c r="C6" s="11">
+        <v>8.4329035573000005E-2</v>
+      </c>
+      <c r="D6" s="16">
+        <v>7.6881148949999997E-3</v>
+      </c>
       <c r="E6" s="20">
         <v>17.800999999999998</v>
       </c>
       <c r="F6" s="20">
         <v>2</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="16"/>
+      <c r="G6" s="11">
+        <v>4.0146823207999997E-2</v>
+      </c>
+      <c r="H6" s="11">
+        <v>3.6574398963E-2</v>
+      </c>
+      <c r="I6" s="16">
+        <v>3.3563730525000002E-3</v>
+      </c>
       <c r="J6" s="23">
         <v>9.7479999999999993</v>
       </c>
       <c r="K6" s="20">
         <v>2</v>
       </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
+      <c r="L6" s="11">
+        <v>3.4905392750999999E-2</v>
+      </c>
+      <c r="M6" s="11">
+        <v>3.1866216822999997E-2</v>
+      </c>
+      <c r="N6" s="11">
+        <v>2.7773169063000001E-3</v>
+      </c>
       <c r="O6" s="20">
         <v>9</v>
       </c>
@@ -24919,27 +24955,45 @@
       <c r="A7" s="20">
         <v>3</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="16"/>
+      <c r="B7" s="11">
+        <v>0.20641670680999999</v>
+      </c>
+      <c r="C7" s="11">
+        <v>0.18738647629999999</v>
+      </c>
+      <c r="D7" s="16">
+        <v>1.7542710528000001E-2</v>
+      </c>
       <c r="E7" s="20">
         <v>47.457999999999998</v>
       </c>
       <c r="F7" s="20">
         <v>3</v>
       </c>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="16"/>
+      <c r="G7" s="11">
+        <v>8.7401050191000001E-2</v>
+      </c>
+      <c r="H7" s="11">
+        <v>7.9684093230999994E-2</v>
+      </c>
+      <c r="I7" s="16">
+        <v>7.3645247068000004E-3</v>
+      </c>
       <c r="J7" s="23">
         <v>16.962</v>
       </c>
       <c r="K7" s="20">
         <v>3</v>
       </c>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
+      <c r="L7" s="11">
+        <v>6.0462507152000002E-2</v>
+      </c>
+      <c r="M7" s="11">
+        <v>5.5129460861999997E-2</v>
+      </c>
+      <c r="N7" s="11">
+        <v>5.0305327304999998E-3</v>
+      </c>
       <c r="O7" s="20">
         <v>12.718999999999999</v>
       </c>
@@ -24952,25 +25006,43 @@
       <c r="A8" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
+      <c r="B8" s="11">
+        <v>0.11220227458</v>
+      </c>
+      <c r="C8" s="11">
+        <v>9.9135661424000002E-2</v>
+      </c>
+      <c r="D8" s="11">
+        <v>9.0466951962999993E-3</v>
+      </c>
       <c r="E8" s="20"/>
       <c r="F8" s="20">
         <v>4</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="16"/>
+      <c r="G8" s="11">
+        <v>0.13530556125000001</v>
+      </c>
+      <c r="H8" s="11">
+        <v>0.12319023664000001</v>
+      </c>
+      <c r="I8" s="16">
+        <v>1.1573918961000001E-2</v>
+      </c>
       <c r="J8" s="23">
         <v>26.009</v>
       </c>
       <c r="K8" s="20">
         <v>4</v>
       </c>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
+      <c r="L8" s="11">
+        <v>8.7424917426000004E-2</v>
+      </c>
+      <c r="M8" s="11">
+        <v>7.9706955125000006E-2</v>
+      </c>
+      <c r="N8" s="11">
+        <v>7.3645247068000004E-3</v>
+      </c>
       <c r="O8" s="20">
         <v>16.966000000000001</v>
       </c>
@@ -24987,18 +25059,30 @@
       <c r="F9" s="20">
         <v>5</v>
       </c>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="16"/>
+      <c r="G9" s="11">
+        <v>0.19196320064</v>
+      </c>
+      <c r="H9" s="11">
+        <v>0.17433660677999999</v>
+      </c>
+      <c r="I9" s="16">
+        <v>1.6677449771999999E-2</v>
+      </c>
       <c r="J9" s="23">
         <v>41.75</v>
       </c>
       <c r="K9" s="20">
         <v>5</v>
       </c>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
+      <c r="L9" s="11">
+        <v>0.10975844803</v>
+      </c>
+      <c r="M9" s="11">
+        <v>0.1001127492</v>
+      </c>
+      <c r="N9" s="11">
+        <v>9.1533049998000007E-3</v>
+      </c>
       <c r="O9" s="20">
         <v>20.881</v>
       </c>
@@ -25015,18 +25099,30 @@
       <c r="F10" s="20">
         <v>6</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="16"/>
+      <c r="G10" s="11">
+        <v>0.24789305111000001</v>
+      </c>
+      <c r="H10" s="11">
+        <v>0.22462702138000001</v>
+      </c>
+      <c r="I10" s="16">
+        <v>2.1129832014E-2</v>
+      </c>
       <c r="J10" s="23">
         <v>72.683000000000007</v>
       </c>
       <c r="K10" s="20">
         <v>6</v>
       </c>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
+      <c r="L10" s="11">
+        <v>0.13044611637</v>
+      </c>
+      <c r="M10" s="11">
+        <v>0.11875805062</v>
+      </c>
+      <c r="N10" s="11">
+        <v>1.1317994305999999E-2</v>
+      </c>
       <c r="O10" s="20">
         <v>24.969000000000001</v>
       </c>
@@ -25043,18 +25139,30 @@
       <c r="F11" s="20">
         <v>7</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="16"/>
+      <c r="G11" s="11">
+        <v>0.29014035373000002</v>
+      </c>
+      <c r="H11" s="11">
+        <v>0.26231390103000002</v>
+      </c>
+      <c r="I11" s="16">
+        <v>2.4378617939000001E-2</v>
+      </c>
       <c r="J11" s="23">
         <v>149.39099999999999</v>
       </c>
       <c r="K11" s="20">
         <v>7</v>
       </c>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
+      <c r="L11" s="11">
+        <v>0.14776341770000001</v>
+      </c>
+      <c r="M11" s="11">
+        <v>0.13440830284999999</v>
+      </c>
+      <c r="N11" s="11">
+        <v>1.2820230534999999E-2</v>
+      </c>
       <c r="O11" s="20">
         <v>28.847999999999999</v>
       </c>
@@ -25071,16 +25179,28 @@
       <c r="F12" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
+      <c r="G12" s="11">
+        <v>0.11364607149</v>
+      </c>
+      <c r="H12" s="11">
+        <v>9.9632884653999998E-2</v>
+      </c>
+      <c r="I12" s="11">
+        <v>9.1533049998000007E-3</v>
+      </c>
       <c r="J12" s="20"/>
       <c r="K12" s="20">
         <v>8</v>
       </c>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
+      <c r="L12" s="11">
+        <v>0.16418154547</v>
+      </c>
+      <c r="M12" s="11">
+        <v>0.14928476476999999</v>
+      </c>
+      <c r="N12" s="11">
+        <v>1.4131744255E-2</v>
+      </c>
       <c r="O12" s="20">
         <v>33.03</v>
       </c>
@@ -25102,9 +25222,15 @@
       <c r="K13" s="20">
         <v>9</v>
       </c>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
+      <c r="L13" s="11">
+        <v>0.17762779110999999</v>
+      </c>
+      <c r="M13" s="11">
+        <v>0.16140146822000001</v>
+      </c>
+      <c r="N13" s="11">
+        <v>1.5416917503E-2</v>
+      </c>
       <c r="O13" s="20">
         <v>36.945</v>
       </c>
@@ -25126,9 +25252,15 @@
       <c r="K14" s="20">
         <v>10</v>
       </c>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
+      <c r="L14" s="11">
+        <v>0.18967492387000001</v>
+      </c>
+      <c r="M14" s="11">
+        <v>0.17229637266</v>
+      </c>
+      <c r="N14" s="11">
+        <v>1.6122962131E-2</v>
+      </c>
       <c r="O14" s="20">
         <v>40.929000000000002</v>
       </c>
@@ -25150,9 +25282,15 @@
       <c r="K15" s="20">
         <v>11</v>
       </c>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
+      <c r="L15" s="11">
+        <v>0.20013582818</v>
+      </c>
+      <c r="M15" s="11">
+        <v>0.18170372106999999</v>
+      </c>
+      <c r="N15" s="11">
+        <v>1.7198547365999999E-2</v>
+      </c>
       <c r="O15" s="20">
         <v>44.854999999999997</v>
       </c>
@@ -25174,9 +25312,15 @@
       <c r="K16" s="20">
         <v>12</v>
       </c>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
+      <c r="L16" s="11">
+        <v>0.21414992911</v>
+      </c>
+      <c r="M16" s="11">
+        <v>0.19431340825000001</v>
+      </c>
+      <c r="N16" s="11">
+        <v>1.8424994133E-2</v>
+      </c>
       <c r="O16" s="20">
         <v>50.978000000000002</v>
       </c>
@@ -25198,9 +25342,15 @@
       <c r="K17" s="20">
         <v>13</v>
       </c>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
+      <c r="L17" s="11">
+        <v>0.23978490613</v>
+      </c>
+      <c r="M17" s="11">
+        <v>0.21735917976999999</v>
+      </c>
+      <c r="N17" s="11">
+        <v>2.0641185842E-2</v>
+      </c>
       <c r="O17" s="20">
         <v>66.174999999999997</v>
       </c>
@@ -25222,9 +25372,15 @@
       <c r="K18" s="20">
         <v>14</v>
       </c>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
+      <c r="L18" s="11">
+        <v>0.26866871197999997</v>
+      </c>
+      <c r="M18" s="11">
+        <v>0.24326044686000001</v>
+      </c>
+      <c r="N18" s="11">
+        <v>2.2777605829E-2</v>
+      </c>
       <c r="O18" s="20">
         <v>96.876000000000005</v>
       </c>
@@ -25246,9 +25402,15 @@
       <c r="K19" s="20">
         <v>15</v>
       </c>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
+      <c r="L19" s="11">
+        <v>0.29014035373000002</v>
+      </c>
+      <c r="M19" s="11">
+        <v>0.26231390103000002</v>
+      </c>
+      <c r="N19" s="11">
+        <v>2.4378617939000001E-2</v>
+      </c>
       <c r="O19" s="20">
         <v>149.39099999999999</v>
       </c>
@@ -25270,9 +25432,15 @@
       <c r="K20" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="L20" s="26"/>
-      <c r="M20" s="26"/>
-      <c r="N20" s="26"/>
+      <c r="L20" s="26">
+        <v>0.11367525186000001</v>
+      </c>
+      <c r="M20" s="26">
+        <v>9.9457650282999993E-2</v>
+      </c>
+      <c r="N20" s="26">
+        <v>9.1533049998000007E-3</v>
+      </c>
       <c r="O20" s="27"/>
       <c r="P20" s="8"/>
       <c r="R20" s="7"/>
@@ -25280,50 +25448,50 @@
       <c r="T20" s="7"/>
     </row>
     <row r="21" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A21" s="44" t="s">
+      <c r="A21" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="45"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="45"/>
-      <c r="O21" s="46"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="37"/>
+      <c r="J21" s="37"/>
+      <c r="K21" s="37"/>
+      <c r="L21" s="37"/>
+      <c r="M21" s="37"/>
+      <c r="N21" s="37"/>
+      <c r="O21" s="38"/>
       <c r="P21" s="29"/>
       <c r="R21" s="30"/>
       <c r="S21" s="30"/>
       <c r="T21" s="30"/>
     </row>
     <row r="22" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47" t="s">
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="47" t="s">
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="47"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
       <c r="R22" s="30"/>
       <c r="S22" s="30"/>
       <c r="T22" s="30"/>
@@ -25382,27 +25550,45 @@
       <c r="A24" s="20">
         <v>1</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
+      <c r="B24" s="11">
+        <v>2.3626998815000001E-2</v>
+      </c>
+      <c r="C24" s="11">
+        <v>2.1539960444999999E-2</v>
+      </c>
+      <c r="D24" s="11">
+        <v>1.8214171592000001E-3</v>
+      </c>
       <c r="E24" s="21">
         <v>7.3890000000000002</v>
       </c>
       <c r="F24" s="11">
         <v>1</v>
       </c>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="16"/>
+      <c r="G24" s="11">
+        <v>1.1981496353E-2</v>
+      </c>
+      <c r="H24" s="11">
+        <v>1.0958819599E-2</v>
+      </c>
+      <c r="I24" s="16">
+        <v>8.1735802136999997E-4</v>
+      </c>
       <c r="J24" s="23">
         <v>5.6689999999999996</v>
       </c>
       <c r="K24" s="20">
         <v>1</v>
       </c>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
+      <c r="L24" s="11">
+        <v>1.1981496353E-2</v>
+      </c>
+      <c r="M24" s="11">
+        <v>1.095882127E-2</v>
+      </c>
+      <c r="N24" s="11">
+        <v>8.1735802136999997E-4</v>
+      </c>
       <c r="O24" s="20">
         <v>5.6689999999999996</v>
       </c>
@@ -25414,27 +25600,45 @@
       <c r="A25" s="20">
         <v>2</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="16"/>
+      <c r="B25" s="11">
+        <v>9.2420607703999999E-2</v>
+      </c>
+      <c r="C25" s="11">
+        <v>8.4243096232999998E-2</v>
+      </c>
+      <c r="D25" s="16">
+        <v>7.6985024198999996E-3</v>
+      </c>
       <c r="E25" s="20">
         <v>17.800999999999998</v>
       </c>
       <c r="F25" s="11">
         <v>2</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="16"/>
+      <c r="G25" s="11">
+        <v>4.0111210841999999E-2</v>
+      </c>
+      <c r="H25" s="11">
+        <v>3.6529865512E-2</v>
+      </c>
+      <c r="I25" s="16">
+        <v>3.2608297727000001E-3</v>
+      </c>
       <c r="J25" s="23">
         <v>9.7479999999999993</v>
       </c>
       <c r="K25" s="20">
         <v>2</v>
       </c>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
+      <c r="L25" s="11">
+        <v>3.4833662304E-2</v>
+      </c>
+      <c r="M25" s="11">
+        <v>3.1818611933999999E-2</v>
+      </c>
+      <c r="N25" s="11">
+        <v>2.6336133289E-3</v>
+      </c>
       <c r="O25" s="20">
         <v>9</v>
       </c>
@@ -25446,27 +25650,45 @@
       <c r="A26" s="20">
         <v>3</v>
       </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="16"/>
+      <c r="B26" s="11">
+        <v>0.20657105717999999</v>
+      </c>
+      <c r="C26" s="11">
+        <v>0.18746347992000001</v>
+      </c>
+      <c r="D26" s="16">
+        <v>1.7951576505E-2</v>
+      </c>
       <c r="E26" s="20">
         <v>47.457999999999998</v>
       </c>
       <c r="F26" s="11">
         <v>3</v>
       </c>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="16"/>
+      <c r="G26" s="11">
+        <v>8.7391513970000001E-2</v>
+      </c>
+      <c r="H26" s="11">
+        <v>7.9600671733999998E-2</v>
+      </c>
+      <c r="I26" s="16">
+        <v>7.4123012437999998E-3</v>
+      </c>
       <c r="J26" s="23">
         <v>16.962</v>
       </c>
       <c r="K26" s="20">
         <v>3</v>
       </c>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
+      <c r="L26" s="11">
+        <v>6.0478338181999998E-2</v>
+      </c>
+      <c r="M26" s="11">
+        <v>5.5216387317000001E-2</v>
+      </c>
+      <c r="N26" s="11">
+        <v>4.7726126054E-3</v>
+      </c>
       <c r="O26" s="20">
         <v>12.718999999999999</v>
       </c>
@@ -25478,25 +25700,43 @@
       <c r="A27" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
+      <c r="B27" s="11">
+        <v>0.11223728502999999</v>
+      </c>
+      <c r="C27" s="11">
+        <v>9.9189707998000004E-2</v>
+      </c>
+      <c r="D27" s="11">
+        <v>9.1782401410000006E-3</v>
+      </c>
       <c r="E27" s="20"/>
       <c r="F27" s="11">
         <v>4</v>
       </c>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="16"/>
+      <c r="G27" s="11">
+        <v>0.13539981976000001</v>
+      </c>
+      <c r="H27" s="11">
+        <v>0.1232908414</v>
+      </c>
+      <c r="I27" s="16">
+        <v>1.1325459531E-2</v>
+      </c>
       <c r="J27" s="23">
         <v>26.009</v>
       </c>
       <c r="K27" s="20">
         <v>4</v>
       </c>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
+      <c r="L27" s="11">
+        <v>8.7415005525000006E-2</v>
+      </c>
+      <c r="M27" s="11">
+        <v>7.9610503316000003E-2</v>
+      </c>
+      <c r="N27" s="11">
+        <v>7.4123012437999998E-3</v>
+      </c>
       <c r="O27" s="20">
         <v>16.966000000000001</v>
       </c>
@@ -25512,18 +25752,30 @@
       <c r="F28" s="11">
         <v>5</v>
       </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="16"/>
+      <c r="G28" s="11">
+        <v>0.19211136517999999</v>
+      </c>
+      <c r="H28" s="11">
+        <v>0.17450410942</v>
+      </c>
+      <c r="I28" s="16">
+        <v>1.6447951836000001E-2</v>
+      </c>
       <c r="J28" s="23">
         <v>41.75</v>
       </c>
       <c r="K28" s="20">
         <v>5</v>
       </c>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
+      <c r="L28" s="11">
+        <v>0.10980555304</v>
+      </c>
+      <c r="M28" s="11">
+        <v>0.10007918145</v>
+      </c>
+      <c r="N28" s="11">
+        <v>9.2179699114000001E-3</v>
+      </c>
       <c r="O28" s="20">
         <v>20.881</v>
       </c>
@@ -25539,18 +25791,30 @@
       <c r="F29" s="11">
         <v>6</v>
       </c>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="16"/>
+      <c r="G29" s="11">
+        <v>0.24800956678</v>
+      </c>
+      <c r="H29" s="11">
+        <v>0.22471394954999999</v>
+      </c>
+      <c r="I29" s="16">
+        <v>2.1329554689E-2</v>
+      </c>
       <c r="J29" s="23">
         <v>72.683000000000007</v>
       </c>
       <c r="K29" s="20">
         <v>6</v>
       </c>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
+      <c r="L29" s="11">
+        <v>0.13048525596999999</v>
+      </c>
+      <c r="M29" s="11">
+        <v>0.11885818707</v>
+      </c>
+      <c r="N29" s="11">
+        <v>1.1119606113000001E-2</v>
+      </c>
       <c r="O29" s="20">
         <v>24.969000000000001</v>
       </c>
@@ -25566,18 +25830,30 @@
       <c r="F30" s="11">
         <v>7</v>
       </c>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="16"/>
+      <c r="G30" s="11">
+        <v>0.29021368147999999</v>
+      </c>
+      <c r="H30" s="11">
+        <v>0.26239849606999999</v>
+      </c>
+      <c r="I30" s="16">
+        <v>2.4513255495E-2</v>
+      </c>
       <c r="J30" s="23">
         <v>149.39099999999999</v>
       </c>
       <c r="K30" s="20">
         <v>7</v>
       </c>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="N30" s="11"/>
+      <c r="L30" s="11">
+        <v>0.14789648762999999</v>
+      </c>
+      <c r="M30" s="11">
+        <v>0.13449537386999999</v>
+      </c>
+      <c r="N30" s="11">
+        <v>1.2798787194999999E-2</v>
+      </c>
       <c r="O30" s="20">
         <v>28.847999999999999</v>
       </c>
@@ -25593,16 +25869,28 @@
       <c r="F31" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
+      <c r="G31" s="11">
+        <v>0.11369435394999999</v>
+      </c>
+      <c r="H31" s="11">
+        <v>9.9735494517999998E-2</v>
+      </c>
+      <c r="I31" s="11">
+        <v>8.6945141600999996E-3</v>
+      </c>
       <c r="J31" s="20"/>
       <c r="K31" s="20">
         <v>8</v>
       </c>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
+      <c r="L31" s="11">
+        <v>0.16430438678000001</v>
+      </c>
+      <c r="M31" s="11">
+        <v>0.14937406315999999</v>
+      </c>
+      <c r="N31" s="11">
+        <v>1.4382275393000001E-2</v>
+      </c>
       <c r="O31" s="20">
         <v>33.03</v>
       </c>
@@ -25623,9 +25911,15 @@
       <c r="K32" s="20">
         <v>9</v>
       </c>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
+      <c r="L32" s="11">
+        <v>0.17775547902</v>
+      </c>
+      <c r="M32" s="11">
+        <v>0.16151022156</v>
+      </c>
+      <c r="N32" s="11">
+        <v>1.5165453987E-2</v>
+      </c>
       <c r="O32" s="20">
         <v>36.945</v>
       </c>
@@ -25646,9 +25940,15 @@
       <c r="K33" s="20">
         <v>10</v>
       </c>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
+      <c r="L33" s="11">
+        <v>0.18983743988999999</v>
+      </c>
+      <c r="M33" s="11">
+        <v>0.17238157936000001</v>
+      </c>
+      <c r="N33" s="11">
+        <v>1.6447951836000001E-2</v>
+      </c>
       <c r="O33" s="20">
         <v>40.929000000000002</v>
       </c>
@@ -25669,9 +25969,15 @@
       <c r="K34" s="20">
         <v>11</v>
       </c>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11"/>
+      <c r="L34" s="11">
+        <v>0.20030843103000001</v>
+      </c>
+      <c r="M34" s="11">
+        <v>0.18190436913999999</v>
+      </c>
+      <c r="N34" s="11">
+        <v>1.6955220787999999E-2</v>
+      </c>
       <c r="O34" s="20">
         <v>44.854999999999997</v>
       </c>
@@ -25692,9 +25998,15 @@
       <c r="K35" s="20">
         <v>12</v>
       </c>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="11"/>
+      <c r="L35" s="11">
+        <v>0.2142858883</v>
+      </c>
+      <c r="M35" s="11">
+        <v>0.19441006473</v>
+      </c>
+      <c r="N35" s="11">
+        <v>1.8447697050999998E-2</v>
+      </c>
       <c r="O35" s="20">
         <v>50.978000000000002</v>
       </c>
@@ -25715,9 +26027,15 @@
       <c r="K36" s="20">
         <v>13</v>
       </c>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11"/>
+      <c r="L36" s="11">
+        <v>0.23990112783</v>
+      </c>
+      <c r="M36" s="11">
+        <v>0.21746068598000001</v>
+      </c>
+      <c r="N36" s="11">
+        <v>2.0385789782000001E-2</v>
+      </c>
       <c r="O36" s="20">
         <v>66.174999999999997</v>
       </c>
@@ -25738,9 +26056,15 @@
       <c r="K37" s="20">
         <v>14</v>
       </c>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
+      <c r="L37" s="11">
+        <v>0.26876263901000003</v>
+      </c>
+      <c r="M37" s="11">
+        <v>0.24335617654</v>
+      </c>
+      <c r="N37" s="11">
+        <v>2.2720423573000002E-2</v>
+      </c>
       <c r="O37" s="20">
         <v>96.876000000000005</v>
       </c>
@@ -25761,9 +26085,15 @@
       <c r="K38" s="20">
         <v>15</v>
       </c>
-      <c r="L38" s="11"/>
-      <c r="M38" s="11"/>
-      <c r="N38" s="11"/>
+      <c r="L38" s="11">
+        <v>0.29021368147999999</v>
+      </c>
+      <c r="M38" s="11">
+        <v>0.26239849606999999</v>
+      </c>
+      <c r="N38" s="11">
+        <v>2.4513255495E-2</v>
+      </c>
       <c r="O38" s="20">
         <v>149.39099999999999</v>
       </c>
@@ -25784,58 +26114,64 @@
       <c r="K39" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="L39" s="26"/>
-      <c r="M39" s="26"/>
-      <c r="N39" s="26"/>
+      <c r="L39" s="26">
+        <v>0.1137193707</v>
+      </c>
+      <c r="M39" s="26">
+        <v>9.9558694335999995E-2</v>
+      </c>
+      <c r="N39" s="26">
+        <v>8.6945141600999996E-3</v>
+      </c>
       <c r="O39" s="27"/>
       <c r="R39" s="7"/>
       <c r="S39" s="7"/>
       <c r="T39" s="7"/>
     </row>
     <row r="40" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A40" s="44" t="s">
+      <c r="A40" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="45"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="45"/>
-      <c r="J40" s="45"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="45"/>
-      <c r="M40" s="45"/>
-      <c r="N40" s="45"/>
-      <c r="O40" s="46"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="37"/>
+      <c r="J40" s="37"/>
+      <c r="K40" s="37"/>
+      <c r="L40" s="37"/>
+      <c r="M40" s="37"/>
+      <c r="N40" s="37"/>
+      <c r="O40" s="38"/>
       <c r="R40" s="30"/>
       <c r="S40" s="30"/>
       <c r="T40" s="30"/>
     </row>
     <row r="41" spans="1:20" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="47"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="47"/>
-      <c r="F41" s="47" t="s">
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="35"/>
+      <c r="F41" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G41" s="47"/>
-      <c r="H41" s="47"/>
-      <c r="I41" s="47"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="47" t="s">
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L41" s="47"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="47"/>
-      <c r="O41" s="47"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="20" t="s">
@@ -25888,27 +26224,45 @@
       <c r="A43" s="20">
         <v>1</v>
       </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
+      <c r="B43" s="11">
+        <v>2.3537362398E-2</v>
+      </c>
+      <c r="C43" s="11">
+        <v>2.1384468401999999E-2</v>
+      </c>
+      <c r="D43" s="11">
+        <v>1.7502554149E-3</v>
+      </c>
       <c r="E43" s="21">
         <v>7.3890000000000002</v>
       </c>
       <c r="F43" s="20">
         <v>1</v>
       </c>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="16"/>
+      <c r="G43" s="11">
+        <v>1.1792768606999999E-2</v>
+      </c>
+      <c r="H43" s="11">
+        <v>1.0816538004999999E-2</v>
+      </c>
+      <c r="I43" s="16">
+        <v>6.4675611433999999E-4</v>
+      </c>
       <c r="J43" s="23">
         <v>5.6689999999999996</v>
       </c>
       <c r="K43" s="20">
         <v>1</v>
       </c>
-      <c r="L43" s="11"/>
-      <c r="M43" s="11"/>
-      <c r="N43" s="11"/>
+      <c r="L43" s="11">
+        <v>1.1792768606999999E-2</v>
+      </c>
+      <c r="M43" s="11">
+        <v>1.0816539529E-2</v>
+      </c>
+      <c r="N43" s="11">
+        <v>6.4675611433999999E-4</v>
+      </c>
       <c r="O43" s="20">
         <v>5.6689999999999996</v>
       </c>
@@ -25917,27 +26271,45 @@
       <c r="A44" s="20">
         <v>2</v>
       </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="16"/>
+      <c r="B44" s="11">
+        <v>9.2487329625000003E-2</v>
+      </c>
+      <c r="C44" s="11">
+        <v>8.4313539150000005E-2</v>
+      </c>
+      <c r="D44" s="16">
+        <v>7.4193272220999997E-3</v>
+      </c>
       <c r="E44" s="20">
         <v>17.800999999999998</v>
       </c>
       <c r="F44" s="20">
         <v>2</v>
       </c>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="16"/>
+      <c r="G44" s="11">
+        <v>3.9900647115999999E-2</v>
+      </c>
+      <c r="H44" s="11">
+        <v>3.6263054431000002E-2</v>
+      </c>
+      <c r="I44" s="16">
+        <v>3.1839389699999999E-3</v>
+      </c>
       <c r="J44" s="23">
         <v>9.7479999999999993</v>
       </c>
       <c r="K44" s="20">
         <v>2</v>
       </c>
-      <c r="L44" s="11"/>
-      <c r="M44" s="11"/>
-      <c r="N44" s="11"/>
+      <c r="L44" s="11">
+        <v>3.4789306196999999E-2</v>
+      </c>
+      <c r="M44" s="11">
+        <v>3.1569979753000001E-2</v>
+      </c>
+      <c r="N44" s="11">
+        <v>2.7916160537E-3</v>
+      </c>
       <c r="O44" s="20">
         <v>9</v>
       </c>
@@ -25946,27 +26318,45 @@
       <c r="A45" s="20">
         <v>3</v>
       </c>
-      <c r="B45" s="11"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="16"/>
+      <c r="B45" s="11">
+        <v>0.20636126406999999</v>
+      </c>
+      <c r="C45" s="11">
+        <v>0.18746975966000001</v>
+      </c>
+      <c r="D45" s="16">
+        <v>1.7452357602E-2</v>
+      </c>
       <c r="E45" s="20">
         <v>47.457999999999998</v>
       </c>
       <c r="F45" s="20">
         <v>3</v>
       </c>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="16"/>
+      <c r="G45" s="11">
+        <v>8.7511468275999996E-2</v>
+      </c>
+      <c r="H45" s="11">
+        <v>7.9774557950000005E-2</v>
+      </c>
+      <c r="I45" s="16">
+        <v>6.9887550692E-3</v>
+      </c>
       <c r="J45" s="23">
         <v>16.962</v>
       </c>
       <c r="K45" s="20">
         <v>3</v>
       </c>
-      <c r="L45" s="11"/>
-      <c r="M45" s="11"/>
-      <c r="N45" s="11"/>
+      <c r="L45" s="11">
+        <v>6.0488137746000002E-2</v>
+      </c>
+      <c r="M45" s="11">
+        <v>5.5083169601000001E-2</v>
+      </c>
+      <c r="N45" s="11">
+        <v>4.8088556939999997E-3</v>
+      </c>
       <c r="O45" s="20">
         <v>12.718999999999999</v>
       </c>
@@ -25975,25 +26365,43 @@
       <c r="A46" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="11"/>
-      <c r="C46" s="11"/>
-      <c r="D46" s="11"/>
+      <c r="B46" s="11">
+        <v>0.11220755323999999</v>
+      </c>
+      <c r="C46" s="11">
+        <v>9.9266861141000001E-2</v>
+      </c>
+      <c r="D46" s="11">
+        <v>9.0345008399999992E-3</v>
+      </c>
       <c r="E46" s="20"/>
       <c r="F46" s="20">
         <v>4</v>
       </c>
-      <c r="G46" s="11"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="16"/>
+      <c r="G46" s="11">
+        <v>0.13534915961999999</v>
+      </c>
+      <c r="H46" s="11">
+        <v>0.12318439874999999</v>
+      </c>
+      <c r="I46" s="16">
+        <v>1.1507771405000001E-2</v>
+      </c>
       <c r="J46" s="23">
         <v>26.009</v>
       </c>
       <c r="K46" s="20">
         <v>4</v>
       </c>
-      <c r="L46" s="11"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="11"/>
+      <c r="L46" s="11">
+        <v>8.7535058025000001E-2</v>
+      </c>
+      <c r="M46" s="11">
+        <v>7.9797130201000002E-2</v>
+      </c>
+      <c r="N46" s="11">
+        <v>6.9887550692E-3</v>
+      </c>
       <c r="O46" s="20">
         <v>16.966000000000001</v>
       </c>
@@ -26006,18 +26414,30 @@
       <c r="F47" s="20">
         <v>5</v>
       </c>
-      <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
-      <c r="I47" s="16"/>
+      <c r="G47" s="11">
+        <v>0.19192090793</v>
+      </c>
+      <c r="H47" s="11">
+        <v>0.17431106000999999</v>
+      </c>
+      <c r="I47" s="16">
+        <v>1.6745319224000001E-2</v>
+      </c>
       <c r="J47" s="23">
         <v>41.75</v>
       </c>
       <c r="K47" s="20">
         <v>5</v>
       </c>
-      <c r="L47" s="11"/>
-      <c r="M47" s="11"/>
-      <c r="N47" s="11"/>
+      <c r="L47" s="11">
+        <v>0.1098233265</v>
+      </c>
+      <c r="M47" s="11">
+        <v>9.9947208669999996E-2</v>
+      </c>
+      <c r="N47" s="11">
+        <v>9.2475222395000008E-3</v>
+      </c>
       <c r="O47" s="20">
         <v>20.881</v>
       </c>
@@ -26030,18 +26450,30 @@
       <c r="F48" s="20">
         <v>6</v>
       </c>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="16"/>
+      <c r="G48" s="11">
+        <v>0.24793296608000001</v>
+      </c>
+      <c r="H48" s="11">
+        <v>0.22480274635</v>
+      </c>
+      <c r="I48" s="16">
+        <v>2.1234353256999999E-2</v>
+      </c>
       <c r="J48" s="23">
         <v>72.683000000000007</v>
       </c>
       <c r="K48" s="20">
         <v>6</v>
       </c>
-      <c r="L48" s="11"/>
-      <c r="M48" s="11"/>
-      <c r="N48" s="11"/>
+      <c r="L48" s="11">
+        <v>0.13043414734</v>
+      </c>
+      <c r="M48" s="11">
+        <v>0.11862544679000001</v>
+      </c>
+      <c r="N48" s="11">
+        <v>1.1236142031999999E-2</v>
+      </c>
       <c r="O48" s="20">
         <v>24.969000000000001</v>
       </c>
@@ -26054,18 +26486,30 @@
       <c r="F49" s="20">
         <v>7</v>
       </c>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="16"/>
+      <c r="G49" s="11">
+        <v>0.29020654143000002</v>
+      </c>
+      <c r="H49" s="11">
+        <v>0.26248864983999998</v>
+      </c>
+      <c r="I49" s="16">
+        <v>2.4478570702000001E-2</v>
+      </c>
       <c r="J49" s="23">
         <v>149.39099999999999</v>
       </c>
       <c r="K49" s="20">
         <v>7</v>
       </c>
-      <c r="L49" s="11"/>
-      <c r="M49" s="11"/>
-      <c r="N49" s="11"/>
+      <c r="L49" s="11">
+        <v>0.14774783736</v>
+      </c>
+      <c r="M49" s="11">
+        <v>0.13456998851999999</v>
+      </c>
+      <c r="N49" s="11">
+        <v>1.2400651168E-2</v>
+      </c>
       <c r="O49" s="20">
         <v>28.847999999999999</v>
       </c>
@@ -26078,16 +26522,28 @@
       <c r="F50" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="11"/>
+      <c r="G50" s="11">
+        <v>0.11360432886000001</v>
+      </c>
+      <c r="H50" s="11">
+        <v>9.9721430042E-2</v>
+      </c>
+      <c r="I50" s="11">
+        <v>9.1337809085000003E-3</v>
+      </c>
       <c r="J50" s="20"/>
       <c r="K50" s="20">
         <v>8</v>
       </c>
-      <c r="L50" s="11"/>
-      <c r="M50" s="11"/>
-      <c r="N50" s="11"/>
+      <c r="L50" s="11">
+        <v>0.16415788346999999</v>
+      </c>
+      <c r="M50" s="11">
+        <v>0.14934620264000001</v>
+      </c>
+      <c r="N50" s="11">
+        <v>1.4190911368000001E-2</v>
+      </c>
       <c r="O50" s="20">
         <v>33.03</v>
       </c>
@@ -26105,9 +26561,15 @@
       <c r="K51" s="20">
         <v>9</v>
       </c>
-      <c r="L51" s="11"/>
-      <c r="M51" s="11"/>
-      <c r="N51" s="11"/>
+      <c r="L51" s="11">
+        <v>0.17761233896</v>
+      </c>
+      <c r="M51" s="11">
+        <v>0.16152573621999999</v>
+      </c>
+      <c r="N51" s="11">
+        <v>1.4925845292000001E-2</v>
+      </c>
       <c r="O51" s="20">
         <v>36.945</v>
       </c>
@@ -26125,9 +26587,15 @@
       <c r="K52" s="20">
         <v>10</v>
       </c>
-      <c r="L52" s="11"/>
-      <c r="M52" s="11"/>
-      <c r="N52" s="11"/>
+      <c r="L52" s="11">
+        <v>0.18965989153000001</v>
+      </c>
+      <c r="M52" s="11">
+        <v>0.17232521410000001</v>
+      </c>
+      <c r="N52" s="11">
+        <v>1.6387848630999999E-2</v>
+      </c>
       <c r="O52" s="20">
         <v>40.929000000000002</v>
       </c>
@@ -26145,9 +26613,15 @@
       <c r="K53" s="20">
         <v>11</v>
       </c>
-      <c r="L53" s="11"/>
-      <c r="M53" s="11"/>
-      <c r="N53" s="11"/>
+      <c r="L53" s="11">
+        <v>0.2001492906</v>
+      </c>
+      <c r="M53" s="11">
+        <v>0.18180854664000001</v>
+      </c>
+      <c r="N53" s="11">
+        <v>1.7100159505E-2</v>
+      </c>
       <c r="O53" s="20">
         <v>44.854999999999997</v>
       </c>
@@ -26165,9 +26639,15 @@
       <c r="K54" s="20">
         <v>12</v>
       </c>
-      <c r="L54" s="11"/>
-      <c r="M54" s="11"/>
-      <c r="N54" s="11"/>
+      <c r="L54" s="11">
+        <v>0.21416779553000001</v>
+      </c>
+      <c r="M54" s="11">
+        <v>0.19451956249999999</v>
+      </c>
+      <c r="N54" s="11">
+        <v>1.7801925592000001E-2</v>
+      </c>
       <c r="O54" s="20">
         <v>50.978000000000002</v>
       </c>
@@ -26185,9 +26665,15 @@
       <c r="K55" s="20">
         <v>13</v>
       </c>
-      <c r="L55" s="11"/>
-      <c r="M55" s="11"/>
-      <c r="N55" s="11"/>
+      <c r="L55" s="11">
+        <v>0.23983670693</v>
+      </c>
+      <c r="M55" s="11">
+        <v>0.21751521449</v>
+      </c>
+      <c r="N55" s="11">
+        <v>2.0218170856000001E-2</v>
+      </c>
       <c r="O55" s="20">
         <v>66.174999999999997</v>
       </c>
@@ -26205,9 +26691,15 @@
       <c r="K56" s="20">
         <v>14</v>
       </c>
-      <c r="L56" s="11"/>
-      <c r="M56" s="11"/>
-      <c r="N56" s="11"/>
+      <c r="L56" s="11">
+        <v>0.26870526557000002</v>
+      </c>
+      <c r="M56" s="11">
+        <v>0.24343065920000001</v>
+      </c>
+      <c r="N56" s="11">
+        <v>2.2878736601E-2</v>
+      </c>
       <c r="O56" s="20">
         <v>96.876000000000005</v>
       </c>
@@ -26225,9 +26717,15 @@
       <c r="K57" s="20">
         <v>15</v>
       </c>
-      <c r="L57" s="11"/>
-      <c r="M57" s="11"/>
-      <c r="N57" s="11"/>
+      <c r="L57" s="11">
+        <v>0.29020654143000002</v>
+      </c>
+      <c r="M57" s="11">
+        <v>0.26248864983999998</v>
+      </c>
+      <c r="N57" s="11">
+        <v>2.4478570702000001E-2</v>
+      </c>
       <c r="O57" s="20">
         <v>149.39099999999999</v>
       </c>
@@ -26245,52 +26743,58 @@
       <c r="K58" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="L58" s="26"/>
-      <c r="M58" s="26"/>
-      <c r="N58" s="26"/>
+      <c r="L58" s="26">
+        <v>0.1136689504</v>
+      </c>
+      <c r="M58" s="26">
+        <v>9.9609957969999996E-2</v>
+      </c>
+      <c r="N58" s="26">
+        <v>8.4893442725999992E-3</v>
+      </c>
       <c r="O58" s="27"/>
     </row>
     <row r="59" spans="1:15" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A59" s="47" t="s">
+      <c r="A59" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="B59" s="47"/>
-      <c r="C59" s="47"/>
-      <c r="D59" s="47"/>
-      <c r="E59" s="47"/>
-      <c r="F59" s="47"/>
-      <c r="G59" s="47"/>
-      <c r="H59" s="47"/>
-      <c r="I59" s="47"/>
-      <c r="J59" s="47"/>
-      <c r="K59" s="47"/>
-      <c r="L59" s="47"/>
-      <c r="M59" s="47"/>
-      <c r="N59" s="47"/>
-      <c r="O59" s="47"/>
+      <c r="B59" s="35"/>
+      <c r="C59" s="35"/>
+      <c r="D59" s="35"/>
+      <c r="E59" s="35"/>
+      <c r="F59" s="35"/>
+      <c r="G59" s="35"/>
+      <c r="H59" s="35"/>
+      <c r="I59" s="35"/>
+      <c r="J59" s="35"/>
+      <c r="K59" s="35"/>
+      <c r="L59" s="35"/>
+      <c r="M59" s="35"/>
+      <c r="N59" s="35"/>
+      <c r="O59" s="35"/>
     </row>
     <row r="60" spans="1:15" s="28" customFormat="1" ht="27" x14ac:dyDescent="0.2">
-      <c r="A60" s="47" t="s">
+      <c r="A60" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B60" s="47"/>
-      <c r="C60" s="47"/>
-      <c r="D60" s="47"/>
-      <c r="E60" s="47"/>
-      <c r="F60" s="47" t="s">
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
+      <c r="D60" s="35"/>
+      <c r="E60" s="35"/>
+      <c r="F60" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G60" s="47"/>
-      <c r="H60" s="47"/>
-      <c r="I60" s="47"/>
-      <c r="J60" s="47"/>
-      <c r="K60" s="47" t="s">
+      <c r="G60" s="35"/>
+      <c r="H60" s="35"/>
+      <c r="I60" s="35"/>
+      <c r="J60" s="35"/>
+      <c r="K60" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L60" s="47"/>
-      <c r="M60" s="47"/>
-      <c r="N60" s="47"/>
-      <c r="O60" s="47"/>
+      <c r="L60" s="35"/>
+      <c r="M60" s="35"/>
+      <c r="N60" s="35"/>
+      <c r="O60" s="35"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61" s="20" t="s">
@@ -26875,6 +27379,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A40:O40"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="F41:J41"/>
+    <mergeCell ref="K41:O41"/>
     <mergeCell ref="A59:O59"/>
     <mergeCell ref="A60:E60"/>
     <mergeCell ref="F60:J60"/>
@@ -26887,11 +27396,6 @@
     <mergeCell ref="F22:J22"/>
     <mergeCell ref="K22:O22"/>
     <mergeCell ref="A21:O21"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A40:O40"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="F41:J41"/>
-    <mergeCell ref="K41:O41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -26923,23 +27427,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
       <c r="P1" s="32"/>
       <c r="Q1" s="32"/>
       <c r="R1" s="32"/>
@@ -27951,23 +28455,23 @@
       <c r="AMJ1" s="32"/>
     </row>
     <row r="2" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
       <c r="P2" s="32"/>
       <c r="Q2" s="32"/>
       <c r="R2" s="32"/>
@@ -28979,27 +29483,27 @@
       <c r="AMJ2" s="32"/>
     </row>
     <row r="3" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
-      <c r="D3" s="47"/>
-      <c r="E3" s="47"/>
-      <c r="F3" s="47" t="s">
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G3" s="47"/>
-      <c r="H3" s="47"/>
-      <c r="I3" s="47"/>
-      <c r="J3" s="47"/>
-      <c r="K3" s="47" t="s">
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
       <c r="P3" s="32"/>
       <c r="Q3" s="32"/>
       <c r="R3" s="22"/>
@@ -30334,23 +30838,23 @@
       <c r="Q20" s="15"/>
     </row>
     <row r="21" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A21" s="47" t="s">
+      <c r="A21" s="35" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="47"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="47"/>
-      <c r="I21" s="47"/>
-      <c r="J21" s="47"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="47"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
+      <c r="G21" s="35"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="35"/>
+      <c r="K21" s="35"/>
+      <c r="L21" s="35"/>
+      <c r="M21" s="35"/>
+      <c r="N21" s="35"/>
+      <c r="O21" s="35"/>
       <c r="P21" s="34"/>
       <c r="Q21" s="34"/>
       <c r="R21" s="32"/>
@@ -31362,27 +31866,27 @@
       <c r="AMJ21" s="32"/>
     </row>
     <row r="22" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="47" t="s">
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="47"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="47"/>
-      <c r="J22" s="47"/>
-      <c r="K22" s="47" t="s">
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L22" s="47"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="47"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
       <c r="P22" s="32"/>
       <c r="Q22" s="32"/>
       <c r="R22" s="32"/>
@@ -32887,23 +33391,23 @@
       <c r="O39" s="25"/>
     </row>
     <row r="40" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A40" s="44" t="s">
+      <c r="A40" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="45"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="45"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="45"/>
-      <c r="I40" s="45"/>
-      <c r="J40" s="45"/>
-      <c r="K40" s="45"/>
-      <c r="L40" s="45"/>
-      <c r="M40" s="45"/>
-      <c r="N40" s="45"/>
-      <c r="O40" s="46"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
+      <c r="E40" s="37"/>
+      <c r="F40" s="37"/>
+      <c r="G40" s="37"/>
+      <c r="H40" s="37"/>
+      <c r="I40" s="37"/>
+      <c r="J40" s="37"/>
+      <c r="K40" s="37"/>
+      <c r="L40" s="37"/>
+      <c r="M40" s="37"/>
+      <c r="N40" s="37"/>
+      <c r="O40" s="38"/>
       <c r="P40" s="32"/>
       <c r="Q40" s="32"/>
       <c r="R40" s="32"/>
@@ -33915,27 +34419,27 @@
       <c r="AMJ40" s="32"/>
     </row>
     <row r="41" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A41" s="47" t="s">
+      <c r="A41" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="47"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="47"/>
-      <c r="F41" s="47" t="s">
+      <c r="B41" s="35"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="35"/>
+      <c r="E41" s="35"/>
+      <c r="F41" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G41" s="47"/>
-      <c r="H41" s="47"/>
-      <c r="I41" s="47"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="47" t="s">
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="35"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L41" s="47"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="47"/>
-      <c r="O41" s="47"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35"/>
+      <c r="N41" s="35"/>
+      <c r="O41" s="35"/>
       <c r="P41" s="32"/>
       <c r="Q41" s="32"/>
       <c r="R41" s="32"/>
@@ -35440,23 +35944,23 @@
       <c r="O58" s="25"/>
     </row>
     <row r="59" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A59" s="44" t="s">
+      <c r="A59" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="45"/>
-      <c r="E59" s="45"/>
-      <c r="F59" s="45"/>
-      <c r="G59" s="45"/>
-      <c r="H59" s="45"/>
-      <c r="I59" s="45"/>
-      <c r="J59" s="45"/>
-      <c r="K59" s="45"/>
-      <c r="L59" s="45"/>
-      <c r="M59" s="45"/>
-      <c r="N59" s="45"/>
-      <c r="O59" s="46"/>
+      <c r="B59" s="37"/>
+      <c r="C59" s="37"/>
+      <c r="D59" s="37"/>
+      <c r="E59" s="37"/>
+      <c r="F59" s="37"/>
+      <c r="G59" s="37"/>
+      <c r="H59" s="37"/>
+      <c r="I59" s="37"/>
+      <c r="J59" s="37"/>
+      <c r="K59" s="37"/>
+      <c r="L59" s="37"/>
+      <c r="M59" s="37"/>
+      <c r="N59" s="37"/>
+      <c r="O59" s="38"/>
       <c r="P59" s="32"/>
       <c r="Q59" s="32"/>
       <c r="R59" s="32"/>
@@ -36468,27 +36972,27 @@
       <c r="AMJ59" s="32"/>
     </row>
     <row r="60" spans="1:1024" s="33" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A60" s="47" t="s">
+      <c r="A60" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="B60" s="47"/>
-      <c r="C60" s="47"/>
-      <c r="D60" s="47"/>
-      <c r="E60" s="47"/>
-      <c r="F60" s="47" t="s">
+      <c r="B60" s="35"/>
+      <c r="C60" s="35"/>
+      <c r="D60" s="35"/>
+      <c r="E60" s="35"/>
+      <c r="F60" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="G60" s="47"/>
-      <c r="H60" s="47"/>
-      <c r="I60" s="47"/>
-      <c r="J60" s="47"/>
-      <c r="K60" s="47" t="s">
+      <c r="G60" s="35"/>
+      <c r="H60" s="35"/>
+      <c r="I60" s="35"/>
+      <c r="J60" s="35"/>
+      <c r="K60" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="L60" s="47"/>
-      <c r="M60" s="47"/>
-      <c r="N60" s="47"/>
-      <c r="O60" s="47"/>
+      <c r="L60" s="35"/>
+      <c r="M60" s="35"/>
+      <c r="N60" s="35"/>
+      <c r="O60" s="35"/>
       <c r="P60" s="32"/>
       <c r="Q60" s="32"/>
       <c r="R60" s="32"/>
@@ -37994,11 +38498,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A60:E60"/>
-    <mergeCell ref="F60:J60"/>
-    <mergeCell ref="K60:O60"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="F41:J41"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A21:O21"/>
@@ -38011,6 +38510,11 @@
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="F3:J3"/>
     <mergeCell ref="K3:O3"/>
+    <mergeCell ref="A60:E60"/>
+    <mergeCell ref="F60:J60"/>
+    <mergeCell ref="K60:O60"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="F41:J41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>